<commit_message>
feat(hierarchy): full-stack support for common-side jigs and symmetrical tooling
</commit_message>
<xml_diff>
--- a/BOM/FA-273 NEW MFG.xlsx
+++ b/BOM/FA-273 NEW MFG.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Darshan Details\Internship Faith Automation\Projects\Spare Part Tracking\SpareTrack\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E01E055-7C18-472A-9161-4796453A53D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E36D344F-FCB6-4EC6-B8F8-B8AA1C65DEBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="476" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="40">
   <si>
     <t>Project Code</t>
   </si>
@@ -121,6 +121,30 @@
   </si>
   <si>
     <t>16</t>
+  </si>
+  <si>
+    <t>LIMORD70</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>17</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>19</t>
+  </si>
+  <si>
+    <t>20</t>
   </si>
 </sst>
 </file>
@@ -735,7 +759,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="C3:H98"/>
+  <dimension ref="C3:H113"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="3" max="3" width="20.33203125" customWidth="1"/>
@@ -2646,6 +2670,217 @@
         <v>1</v>
       </c>
     </row>
+    <row r="99" spans="3:8" ht="21.6" thickBot="1">
+      <c r="D99" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="E99" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="F99" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="G99" s="17"/>
+      <c r="H99" s="19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="100" spans="3:8" ht="21.6" thickBot="1">
+      <c r="D100" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="E100" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="F100" s="22" t="s">
+        <v>14</v>
+      </c>
+      <c r="H100" s="19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="101" spans="3:8" ht="21.6" thickBot="1">
+      <c r="D101" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="E101" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="F101" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="H101" s="19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="102" spans="3:8" ht="21.6" thickBot="1">
+      <c r="D102" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="E102" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="F102" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="H102" s="19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="103" spans="3:8" ht="21.6" thickBot="1">
+      <c r="D103" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="E103" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="F103" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="H103" s="19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="104" spans="3:8" ht="21.6" thickBot="1">
+      <c r="D104" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="E104" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="F104" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="H104" s="19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="105" spans="3:8" ht="21.6" thickBot="1">
+      <c r="D105" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="E105" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="F105" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="H105" s="19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="106" spans="3:8" ht="21.6" thickBot="1">
+      <c r="D106" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="E106" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="F106" s="22" t="s">
+        <v>33</v>
+      </c>
+      <c r="H106" s="19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="107" spans="3:8" ht="21.6" thickBot="1">
+      <c r="D107" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="E107" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="F107" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="H107" s="19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="108" spans="3:8" ht="21.6" thickBot="1">
+      <c r="D108" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="E108" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="F108" s="22" t="s">
+        <v>35</v>
+      </c>
+      <c r="H108" s="19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="109" spans="3:8" ht="21.6" thickBot="1">
+      <c r="D109" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="E109" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="F109" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="H109" s="19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="110" spans="3:8" ht="21.6" thickBot="1">
+      <c r="D110" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="E110" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="F110" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="H110" s="19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="111" spans="3:8" ht="21.6" thickBot="1">
+      <c r="D111" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="E111" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="F111" s="22" t="s">
+        <v>37</v>
+      </c>
+      <c r="H111" s="19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="112" spans="3:8" ht="21.6" thickBot="1">
+      <c r="D112" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="E112" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="F112" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="H112" s="19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="113" spans="4:8" ht="21.6" thickBot="1">
+      <c r="D113" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="E113" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="F113" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="H113" s="19">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>